<commit_message>
Repeat instructions until the "I was told" question is correct; add Tab skip
Comprehension check:
- Wrap instruct_introduction -> instruct_questions -> new instruct_incorrect
  routine in a <condition>_comprehension loop (control, up, down). A wrong
  answer shows an "answered incorrectly" page, then the instructions and
  questions again, until the answer is correct.
- instruct_questions End Routine compares the slider label with a new
  toldCorrect column in the six instructions_*.xlsx files (control: Have no
  effect on, up: Improve, down: Impair) and saves told_correct per attempt.

Wording:
- "I was told" slider: Hinder -> Impair, to match the down instructions.
- Belief sliders (baseline and instructions): Greatly hinders -> Greatly impairs.

Piloting:
- tab_skip_code: in pilot mode, Tab ends the current routine.
- runMode saved as Pilot from Builder.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/experiment/task/instructions_strategy_control.xlsx
+++ b/experiment/task/instructions_strategy_control.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,13 +413,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
           <t>instructionText</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>toldCorrect</t>
         </is>
       </c>
     </row>
@@ -432,6 +437,11 @@
 You do not need to do anything in particular while watching. Simply watch each video as you normally would, and pay attention to what happens in it.</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Have no effect on</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>